<commit_message>
Updated MEX model - 2026-04-22 22:18
</commit_message>
<xml_diff>
--- a/VerveStacks_MEX/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_MEX/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_MEX\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{33348B94-3088-4E18-BCD9-581E46FDAA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4324227D-3A4A-41FB-988D-A596AA21CE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="604">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -1936,6 +1936,9 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>e_MX13-400_MEX,e_MX22-400_MEX,e_MX47-400_MEX,e_MX59-400_MEX,e_MX64-400_MEX,e_MX65-400_MEX,e_r16016425-400_MEX,e_w100657593-400_MEX,e_w1119978083-400_MEX,e_w113005842-400_MEX,e_w1181050521-400_MEX,e_w1376647652-400_MEX,e_w318948686-400_MEX,e_w320586165-400_MEX,e_w322722579-400_MEX,e_w324339640-400_MEX,e_w325906414-400_MEX,e_w328454682-400_MEX,e_w764377660-400_MEX</t>
   </si>
 </sst>
 </file>
@@ -3832,7 +3835,7 @@
       </c>
       <c r="L27" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_MX13-400_MEX,e_MX22-400_MEX,e_MX47-400_MEX,e_MX59-400_MEX,e_MX64-400_MEX,e_MX65-400_MEX,e_r16016425-400_MEX,e_w100657593-400_MEX,e_w1119978083-400_MEX,e_w113005842-400_MEX,e_w1181050521-400_MEX,e_w1376647652-400_MEX,e_w318948686-400_MEX,e_w320586165-400_MEX,e_w322722579-400_MEX,e_w324339640-400_MEX,e_w325906414-400_MEX,e_w328454682-400_MEX,e_w764377660-400_MEX</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -3854,7 +3857,7 @@
       </c>
       <c r="K28" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_MX13-400_MEX,e_MX22-400_MEX,e_MX47-400_MEX,e_MX59-400_MEX,e_MX64-400_MEX,e_MX65-400_MEX,e_r16016425-400_MEX,e_w100657593-400_MEX,e_w1119978083-400_MEX,e_w113005842-400_MEX,e_w1181050521-400_MEX,e_w1376647652-400_MEX,e_w318948686-400_MEX,e_w320586165-400_MEX,e_w322722579-400_MEX,e_w324339640-400_MEX,e_w325906414-400_MEX,e_w328454682-400_MEX,e_w764377660-400_MEX</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -3869,7 +3872,7 @@
         <v>50</v>
       </c>
       <c r="V28" s="147" t="s">
-        <v>19</v>
+        <v>603</v>
       </c>
     </row>
   </sheetData>
@@ -6670,7 +6673,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF9E8222-9DEC-4098-83CD-3A887557DCDC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AAB9931-1541-4579-8421-138A95D3FF54}">
   <dimension ref="B9:M69"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8788,7 +8791,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{421ABD44-5257-4B0A-9CF7-D77C69103E92}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CEB42CB-B599-4129-BEB9-ED389B1AB3E4}">
   <dimension ref="B9:Z54"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -11410,7 +11413,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF40B7C-8A21-4599-916A-C966B8D30BFE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{348BDD94-8563-4E36-A167-4FBA22E8443D}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated MEX model - 2026-04-23 00:11
</commit_message>
<xml_diff>
--- a/VerveStacks_MEX/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_MEX/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_MEX\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4324227D-3A4A-41FB-988D-A596AA21CE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{666F5BEA-FA3A-4D11-B4B5-756271183ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="603">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -1936,9 +1936,6 @@
   </si>
   <si>
     <t>yes</t>
-  </si>
-  <si>
-    <t>e_MX13-400_MEX,e_MX22-400_MEX,e_MX47-400_MEX,e_MX59-400_MEX,e_MX64-400_MEX,e_MX65-400_MEX,e_r16016425-400_MEX,e_w100657593-400_MEX,e_w1119978083-400_MEX,e_w113005842-400_MEX,e_w1181050521-400_MEX,e_w1376647652-400_MEX,e_w318948686-400_MEX,e_w320586165-400_MEX,e_w322722579-400_MEX,e_w324339640-400_MEX,e_w325906414-400_MEX,e_w328454682-400_MEX,e_w764377660-400_MEX</t>
   </si>
 </sst>
 </file>
@@ -3835,7 +3832,7 @@
       </c>
       <c r="L27" t="str">
         <f>$V$28</f>
-        <v>e_MX13-400_MEX,e_MX22-400_MEX,e_MX47-400_MEX,e_MX59-400_MEX,e_MX64-400_MEX,e_MX65-400_MEX,e_r16016425-400_MEX,e_w100657593-400_MEX,e_w1119978083-400_MEX,e_w113005842-400_MEX,e_w1181050521-400_MEX,e_w1376647652-400_MEX,e_w318948686-400_MEX,e_w320586165-400_MEX,e_w322722579-400_MEX,e_w324339640-400_MEX,e_w325906414-400_MEX,e_w328454682-400_MEX,e_w764377660-400_MEX</v>
+        <v>ELC</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -3857,7 +3854,7 @@
       </c>
       <c r="K28" t="str">
         <f>$V$28</f>
-        <v>e_MX13-400_MEX,e_MX22-400_MEX,e_MX47-400_MEX,e_MX59-400_MEX,e_MX64-400_MEX,e_MX65-400_MEX,e_r16016425-400_MEX,e_w100657593-400_MEX,e_w1119978083-400_MEX,e_w113005842-400_MEX,e_w1181050521-400_MEX,e_w1376647652-400_MEX,e_w318948686-400_MEX,e_w320586165-400_MEX,e_w322722579-400_MEX,e_w324339640-400_MEX,e_w325906414-400_MEX,e_w328454682-400_MEX,e_w764377660-400_MEX</v>
+        <v>ELC</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -3872,7 +3869,7 @@
         <v>50</v>
       </c>
       <c r="V28" s="147" t="s">
-        <v>603</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -6673,7 +6670,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AAB9931-1541-4579-8421-138A95D3FF54}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C77C47A6-9015-4BA4-9767-04F2E03FC2E0}">
   <dimension ref="B9:M69"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8791,7 +8788,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CEB42CB-B599-4129-BEB9-ED389B1AB3E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AAE1F6C-AF5E-47C6-8FC9-4CA849F2F034}">
   <dimension ref="B9:Z54"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -11413,7 +11410,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{348BDD94-8563-4E36-A167-4FBA22E8443D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1C74C42-D628-4AC6-AB49-0FDFC146E4DF}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>